<commit_message>
Updated with comments for video links.
</commit_message>
<xml_diff>
--- a/144/DQ Templates and Instructions/Topic 1 DQ 1/Topic 1 DQ 1.xlsx
+++ b/144/DQ Templates and Instructions/Topic 1 DQ 1/Topic 1 DQ 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gcumail.sharepoint.com/sites/MathematicsProgramFacultyStaff-MATOFTF/Shared Documents/MATOFTF/ALEKS/DQ Templates and Instructions/Topic 1 DQ 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="120" documentId="8_{197DFB2F-3D6E-4006-9337-6C654C7D47B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3345079F-C7E7-4C14-BB93-8889B4589617}"/>
+  <xr:revisionPtr revIDLastSave="124" documentId="8_{197DFB2F-3D6E-4006-9337-6C654C7D47B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{351851BE-7648-408A-95BF-C14B0DF02E34}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{4FCF7FA6-22BB-4545-AB27-D5B8AACA448D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4FCF7FA6-22BB-4545-AB27-D5B8AACA448D}"/>
   </bookViews>
   <sheets>
     <sheet name="Goals and Instructions" sheetId="4" r:id="rId1"/>
@@ -45,6 +45,33 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={70924595-1501-455D-AEAD-D19C623E0B48}</author>
+    <author>tc={4D01F969-C016-49F1-B66A-E0F61BFB82DD}</author>
+  </authors>
+  <commentList>
+    <comment ref="C2" authorId="0" shapeId="0" xr:uid="{70924595-1501-455D-AEAD-D19C623E0B48}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    https://www.loom.com/share/7afe56992a4045b6ba3c4ce50c5dc624</t>
+      </text>
+    </comment>
+    <comment ref="C3" authorId="1" shapeId="0" xr:uid="{4D01F969-C016-49F1-B66A-E0F61BFB82DD}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    https://www.loom.com/share/2b55793d438c4e3ea60bd6fe69b70766?sid=ea386e71-e314-48ad-9076-167dbf41817d</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
@@ -442,7 +469,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode=";;;"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -568,6 +595,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -1486,6 +1519,88 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1504,41 +1619,43 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" indent="1"/>
@@ -1568,167 +1685,41 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="36" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="37" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1756,6 +1747,24 @@
     <xf numFmtId="0" fontId="9" fillId="12" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
@@ -1764,6 +1773,30 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1962,6 +1995,12 @@
     <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Richard Ketchersid" id="{E1965639-C3B0-4AA7-85E7-35B439D24F6F}" userId="S::richard.ketchersid@gcu.edu::a14ec2f7-27bd-40c3-90d9-209834cdef57" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2259,6 +2298,29 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="C2" dT="2026-07-16T19:26:47.87" personId="{E1965639-C3B0-4AA7-85E7-35B439D24F6F}" id="{70924595-1501-455D-AEAD-D19C623E0B48}">
+    <text>https://www.loom.com/share/7afe56992a4045b6ba3c4ce50c5dc624</text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>2011169662</xltc2:checksum>
+        <xltc2:hyperlink startIndex="0" length="59" url="https://www.loom.com/share/7afe56992a4045b6ba3c4ce50c5dc624"/>
+      </x:ext>
+    </extLst>
+  </threadedComment>
+  <threadedComment ref="C3" dT="2026-07-16T19:27:08.18" personId="{E1965639-C3B0-4AA7-85E7-35B439D24F6F}" id="{4D01F969-C016-49F1-B66A-E0F61BFB82DD}">
+    <text>https://www.loom.com/share/2b55793d438c4e3ea60bd6fe69b70766?sid=ea386e71-e314-48ad-9076-167dbf41817d</text>
+    <extLst>
+      <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
+        <xltc2:checksum>4113386665</xltc2:checksum>
+        <xltc2:hyperlink startIndex="0" length="100" url="https://www.loom.com/share/2b55793d438c4e3ea60bd6fe69b70766?sid=ea386e71-e314-48ad-9076-167dbf41817d"/>
+      </x:ext>
+    </extLst>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{329EF0F7-756C-4FB0-8A3F-8C263248E1C8}">
   <dimension ref="B2:J18"/>
@@ -2443,7 +2505,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7870B2E2-92BC-47AC-B93B-26715350F717}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7870B2E2-92BC-47AC-B93B-26715350F717}">
   <dimension ref="A1:O28"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2466,94 +2528,94 @@
       <c r="A1" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="147" t="str">
+      <c r="L1" s="107" t="str">
         <f ca="1">IF(OR(I2="Excel Desktop",I2="Excel Online"),"","You are not using Excel, please proceed to office.com, log in with your GCU credentials, and install the current Office 365, or use the online versions. Work not completed in Excel must be redone.")</f>
         <v/>
       </c>
-      <c r="M1" s="148"/>
-      <c r="N1" s="148"/>
-      <c r="O1" s="149"/>
+      <c r="M1" s="108"/>
+      <c r="N1" s="108"/>
+      <c r="O1" s="109"/>
     </row>
     <row r="2" spans="1:15" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B2" s="31"/>
-      <c r="C2" s="141" t="s">
+      <c r="C2" s="101" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="142"/>
-      <c r="E2" s="143"/>
+      <c r="D2" s="102"/>
+      <c r="E2" s="103"/>
       <c r="G2" s="29" t="s">
         <v>14</v>
       </c>
       <c r="H2" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="I2" s="139" t="str" cm="1">
+      <c r="I2" s="99" t="str" cm="1">
         <f t="array" aca="1" ref="I2" ca="1">checksys()</f>
         <v>Excel Desktop</v>
       </c>
-      <c r="J2" s="140"/>
-      <c r="L2" s="150"/>
-      <c r="M2" s="151"/>
-      <c r="N2" s="151"/>
-      <c r="O2" s="152"/>
+      <c r="J2" s="100"/>
+      <c r="L2" s="110"/>
+      <c r="M2" s="111"/>
+      <c r="N2" s="111"/>
+      <c r="O2" s="112"/>
     </row>
     <row r="3" spans="1:15" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="31"/>
-      <c r="C3" s="141" t="s">
+      <c r="C3" s="101" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="142"/>
-      <c r="E3" s="143"/>
-      <c r="L3" s="153"/>
-      <c r="M3" s="154"/>
-      <c r="N3" s="154"/>
-      <c r="O3" s="155"/>
+      <c r="D3" s="102"/>
+      <c r="E3" s="103"/>
+      <c r="L3" s="113"/>
+      <c r="M3" s="114"/>
+      <c r="N3" s="114"/>
+      <c r="O3" s="115"/>
     </row>
     <row r="4" spans="1:15" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="94" t="s">
+      <c r="B4" s="120" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="95"/>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="96"/>
-      <c r="M4" s="136" t="s">
+      <c r="C4" s="121"/>
+      <c r="D4" s="121"/>
+      <c r="E4" s="121"/>
+      <c r="F4" s="122"/>
+      <c r="M4" s="96" t="s">
         <v>10</v>
       </c>
-      <c r="N4" s="137"/>
+      <c r="N4" s="97"/>
     </row>
     <row r="5" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="97"/>
-      <c r="C5" s="98"/>
-      <c r="D5" s="98"/>
-      <c r="E5" s="98"/>
-      <c r="F5" s="99"/>
-      <c r="M5" s="138" t="s">
+      <c r="B5" s="123"/>
+      <c r="C5" s="124"/>
+      <c r="D5" s="124"/>
+      <c r="E5" s="124"/>
+      <c r="F5" s="125"/>
+      <c r="M5" s="98" t="s">
         <v>11</v>
       </c>
-      <c r="N5" s="138"/>
+      <c r="N5" s="98"/>
     </row>
     <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B6" s="122" t="s">
+      <c r="B6" s="126" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="123"/>
-      <c r="D6" s="103" t="s">
+      <c r="C6" s="127"/>
+      <c r="D6" s="149" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="105" t="s">
+      <c r="E6" s="151" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="132" t="s">
+      <c r="F6" s="136" t="s">
         <v>20</v>
       </c>
-      <c r="G6" s="110" t="s">
+      <c r="G6" s="156" t="s">
         <v>21</v>
       </c>
-      <c r="I6" s="124" t="s">
+      <c r="I6" s="128" t="s">
         <v>22</v>
       </c>
-      <c r="J6" s="125"/>
+      <c r="J6" s="129"/>
     </row>
     <row r="7" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
@@ -2562,10 +2624,10 @@
       <c r="C7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="104"/>
-      <c r="E7" s="106"/>
-      <c r="F7" s="133"/>
-      <c r="G7" s="111"/>
+      <c r="D7" s="150"/>
+      <c r="E7" s="152"/>
+      <c r="F7" s="137"/>
+      <c r="G7" s="157"/>
       <c r="I7" s="18" t="s">
         <v>25</v>
       </c>
@@ -2594,10 +2656,10 @@
       </c>
     </row>
     <row r="9" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="126" t="s">
+      <c r="B9" s="130" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="127"/>
+      <c r="C9" s="131"/>
       <c r="D9" s="2" t="s">
         <v>33</v>
       </c>
@@ -2616,8 +2678,8 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="128"/>
-      <c r="C10" s="129"/>
+      <c r="B10" s="132"/>
+      <c r="C10" s="133"/>
       <c r="D10" s="2" t="s">
         <v>38</v>
       </c>
@@ -2636,8 +2698,8 @@
       </c>
     </row>
     <row r="11" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="128"/>
-      <c r="C11" s="129"/>
+      <c r="B11" s="132"/>
+      <c r="C11" s="133"/>
       <c r="D11" s="2" t="s">
         <v>43</v>
       </c>
@@ -2656,8 +2718,8 @@
       </c>
     </row>
     <row r="12" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="130"/>
-      <c r="C12" s="131"/>
+      <c r="B12" s="134"/>
+      <c r="C12" s="135"/>
       <c r="D12" s="7" t="s">
         <v>48</v>
       </c>
@@ -2670,19 +2732,19 @@
       </c>
     </row>
     <row r="13" spans="1:15" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="107" t="s">
+      <c r="B13" s="153" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="108"/>
-      <c r="D13" s="108"/>
-      <c r="E13" s="108"/>
-      <c r="F13" s="109"/>
-      <c r="I13" s="144" t="s">
+      <c r="C13" s="154"/>
+      <c r="D13" s="154"/>
+      <c r="E13" s="154"/>
+      <c r="F13" s="155"/>
+      <c r="I13" s="104" t="s">
         <v>52</v>
       </c>
-      <c r="J13" s="145"/>
-      <c r="K13" s="145"/>
-      <c r="L13" s="146"/>
+      <c r="J13" s="105"/>
+      <c r="K13" s="105"/>
+      <c r="L13" s="106"/>
     </row>
     <row r="14" spans="1:15" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="42"/>
@@ -2693,17 +2755,17 @@
       <c r="H14" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="I14" s="156" t="s">
+      <c r="I14" s="116" t="s">
         <v>54</v>
       </c>
-      <c r="J14" s="156"/>
-      <c r="K14" s="156"/>
-      <c r="L14" s="157"/>
-      <c r="M14" s="134" t="s">
+      <c r="J14" s="116"/>
+      <c r="K14" s="116"/>
+      <c r="L14" s="117"/>
+      <c r="M14" s="94" t="s">
         <v>55</v>
       </c>
-      <c r="N14" s="135"/>
-      <c r="O14" s="135"/>
+      <c r="N14" s="95"/>
+      <c r="O14" s="95"/>
     </row>
     <row r="15" spans="1:15" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="13"/>
@@ -2712,12 +2774,12 @@
       <c r="H15" s="35">
         <v>15</v>
       </c>
-      <c r="I15" s="120" t="s">
+      <c r="I15" s="118" t="s">
         <v>56</v>
       </c>
-      <c r="J15" s="120"/>
-      <c r="K15" s="120"/>
-      <c r="L15" s="121"/>
+      <c r="J15" s="118"/>
+      <c r="K15" s="118"/>
+      <c r="L15" s="119"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B16" s="13"/>
@@ -2726,47 +2788,47 @@
       <c r="H16" s="27">
         <v>16</v>
       </c>
-      <c r="I16" s="112" t="s">
+      <c r="I16" s="138" t="s">
         <v>57</v>
       </c>
-      <c r="J16" s="112"/>
-      <c r="K16" s="112"/>
-      <c r="L16" s="113"/>
+      <c r="J16" s="138"/>
+      <c r="K16" s="138"/>
+      <c r="L16" s="139"/>
     </row>
     <row r="17" spans="2:12" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="12"/>
       <c r="H17" s="28">
         <v>16</v>
       </c>
-      <c r="I17" s="114" t="s">
+      <c r="I17" s="140" t="s">
         <v>58</v>
       </c>
-      <c r="J17" s="114"/>
-      <c r="K17" s="114"/>
-      <c r="L17" s="115"/>
+      <c r="J17" s="140"/>
+      <c r="K17" s="140"/>
+      <c r="L17" s="141"/>
     </row>
     <row r="18" spans="2:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="94" t="s">
+      <c r="B18" s="120" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="95"/>
-      <c r="D18" s="95"/>
-      <c r="E18" s="95"/>
-      <c r="F18" s="96"/>
+      <c r="C18" s="121"/>
+      <c r="D18" s="121"/>
+      <c r="E18" s="121"/>
+      <c r="F18" s="122"/>
     </row>
     <row r="19" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="97"/>
-      <c r="C19" s="98"/>
-      <c r="D19" s="98"/>
-      <c r="E19" s="98"/>
-      <c r="F19" s="99"/>
+      <c r="B19" s="123"/>
+      <c r="C19" s="124"/>
+      <c r="D19" s="124"/>
+      <c r="E19" s="124"/>
+      <c r="F19" s="125"/>
     </row>
     <row r="20" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="100" t="s">
+      <c r="B20" s="146" t="s">
         <v>80</v>
       </c>
-      <c r="C20" s="100"/>
-      <c r="D20" s="100"/>
+      <c r="C20" s="146"/>
+      <c r="D20" s="146"/>
       <c r="E20" s="10" t="s">
         <v>60</v>
       </c>
@@ -2777,15 +2839,15 @@
         <v>62</v>
       </c>
       <c r="H20" s="17"/>
-      <c r="I20" s="118" t="s">
+      <c r="I20" s="144" t="s">
         <v>63</v>
       </c>
-      <c r="J20" s="119"/>
+      <c r="J20" s="145"/>
     </row>
     <row r="21" spans="2:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="101"/>
-      <c r="C21" s="101"/>
-      <c r="D21" s="101"/>
+      <c r="B21" s="147"/>
+      <c r="C21" s="147"/>
+      <c r="D21" s="147"/>
       <c r="E21" s="33"/>
       <c r="F21" s="2" t="s">
         <v>64</v>
@@ -2794,15 +2856,15 @@
         <v>65</v>
       </c>
       <c r="H21" s="41"/>
-      <c r="I21" s="116" t="s">
+      <c r="I21" s="142" t="s">
         <v>66</v>
       </c>
-      <c r="J21" s="116"/>
+      <c r="J21" s="142"/>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B22" s="101"/>
-      <c r="C22" s="101"/>
-      <c r="D22" s="101"/>
+      <c r="B22" s="147"/>
+      <c r="C22" s="147"/>
+      <c r="D22" s="147"/>
       <c r="E22" s="33"/>
       <c r="F22" s="2" t="s">
         <v>67</v>
@@ -2811,15 +2873,15 @@
         <v>68</v>
       </c>
       <c r="H22" s="41"/>
-      <c r="I22" s="117" t="s">
+      <c r="I22" s="143" t="s">
         <v>69</v>
       </c>
-      <c r="J22" s="117"/>
+      <c r="J22" s="143"/>
     </row>
     <row r="23" spans="2:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="101"/>
-      <c r="C23" s="101"/>
-      <c r="D23" s="101"/>
+      <c r="B23" s="147"/>
+      <c r="C23" s="147"/>
+      <c r="D23" s="147"/>
       <c r="E23" s="33"/>
       <c r="F23" s="2" t="s">
         <v>70</v>
@@ -2828,71 +2890,90 @@
         <v>71</v>
       </c>
       <c r="H23" s="41"/>
-      <c r="I23" s="117" t="s">
+      <c r="I23" s="143" t="s">
         <v>72</v>
       </c>
-      <c r="J23" s="117"/>
+      <c r="J23" s="143"/>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B24" s="101"/>
-      <c r="C24" s="101"/>
-      <c r="D24" s="101"/>
+      <c r="B24" s="147"/>
+      <c r="C24" s="147"/>
+      <c r="D24" s="147"/>
       <c r="E24" s="33"/>
-      <c r="F24" s="102" t="s">
+      <c r="F24" s="148" t="s">
         <v>73</v>
       </c>
-      <c r="G24" s="102"/>
+      <c r="G24" s="148"/>
       <c r="H24" s="36"/>
       <c r="I24" s="37"/>
       <c r="J24" s="37"/>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B25" s="101"/>
-      <c r="C25" s="101"/>
-      <c r="D25" s="101"/>
+      <c r="B25" s="147"/>
+      <c r="C25" s="147"/>
+      <c r="D25" s="147"/>
       <c r="E25" s="33"/>
-      <c r="F25" s="102"/>
-      <c r="G25" s="102"/>
+      <c r="F25" s="148"/>
+      <c r="G25" s="148"/>
       <c r="H25" s="38"/>
       <c r="I25" s="39"/>
       <c r="J25" s="39"/>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B26" s="101"/>
-      <c r="C26" s="101"/>
-      <c r="D26" s="101"/>
+      <c r="B26" s="147"/>
+      <c r="C26" s="147"/>
+      <c r="D26" s="147"/>
       <c r="E26" s="33"/>
-      <c r="F26" s="102"/>
-      <c r="G26" s="102"/>
+      <c r="F26" s="148"/>
+      <c r="G26" s="148"/>
       <c r="H26" s="38"/>
       <c r="I26" s="39"/>
       <c r="J26" s="39"/>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B27" s="101"/>
-      <c r="C27" s="101"/>
-      <c r="D27" s="101"/>
+      <c r="B27" s="147"/>
+      <c r="C27" s="147"/>
+      <c r="D27" s="147"/>
       <c r="E27" s="33"/>
-      <c r="F27" s="102"/>
-      <c r="G27" s="102"/>
+      <c r="F27" s="148"/>
+      <c r="G27" s="148"/>
       <c r="H27" s="38"/>
       <c r="I27" s="39"/>
       <c r="J27" s="39"/>
     </row>
     <row r="28" spans="2:12" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="101"/>
-      <c r="C28" s="101"/>
-      <c r="D28" s="101"/>
+      <c r="B28" s="147"/>
+      <c r="C28" s="147"/>
+      <c r="D28" s="147"/>
       <c r="E28" s="33"/>
-      <c r="F28" s="102"/>
-      <c r="G28" s="102"/>
+      <c r="F28" s="148"/>
+      <c r="G28" s="148"/>
       <c r="H28" s="38"/>
       <c r="I28" s="39"/>
       <c r="J28" s="39"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="SvKos635J1JsYx1ldicBdy9fqj4eL2Oy4nZQGHq+duRaGU3MFkYZYUAxS00iFZu3BKiyhvGgFuv0/tV7SpGqOA==" saltValue="vl0rh4dSrBvr/sYKmw7oOA==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="BLIAlMBPgqH+NPEse4s68RjHq+iBp2ZxiPwbr85ja6anELCVKxbZV0o63eupwo+XV0ZheD91KVylaqjLC4V1wA==" saltValue="5R/Fmu0ewxRZ2Clu6FEY8g==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="28">
+    <mergeCell ref="B18:F19"/>
+    <mergeCell ref="B20:D28"/>
+    <mergeCell ref="F24:G28"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="I16:L16"/>
+    <mergeCell ref="I17:L17"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="I15:L15"/>
+    <mergeCell ref="B4:F5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="B9:C12"/>
+    <mergeCell ref="F6:F7"/>
     <mergeCell ref="M14:O14"/>
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="M5:N5"/>
@@ -2902,25 +2983,6 @@
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="L1:O3"/>
     <mergeCell ref="I14:L14"/>
-    <mergeCell ref="I15:L15"/>
-    <mergeCell ref="B4:F5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="B9:C12"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="I16:L16"/>
-    <mergeCell ref="I17:L17"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="B18:F19"/>
-    <mergeCell ref="B20:D28"/>
-    <mergeCell ref="F24:G28"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="G6:G7"/>
   </mergeCells>
   <conditionalFormatting sqref="B8:C8 F8:F12 H21:H23 E21:E28">
     <cfRule type="expression" dxfId="10" priority="1">
@@ -2950,6 +3012,7 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId5"/>
+  <legacyDrawing r:id="rId6"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -3070,13 +3133,13 @@
   <sheetData>
     <row r="1" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B2" s="158" t="s">
+      <c r="B2" s="166" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="159"/>
-      <c r="D2" s="159"/>
-      <c r="E2" s="159"/>
-      <c r="F2" s="160"/>
+      <c r="C2" s="167"/>
+      <c r="D2" s="167"/>
+      <c r="E2" s="167"/>
+      <c r="F2" s="168"/>
       <c r="L2" s="46">
         <v>1</v>
       </c>
@@ -3093,11 +3156,11 @@
       </c>
     </row>
     <row r="3" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="161"/>
-      <c r="C3" s="162"/>
-      <c r="D3" s="162"/>
-      <c r="E3" s="162"/>
-      <c r="F3" s="163"/>
+      <c r="B3" s="169"/>
+      <c r="C3" s="170"/>
+      <c r="D3" s="170"/>
+      <c r="E3" s="170"/>
+      <c r="F3" s="171"/>
       <c r="L3" s="46">
         <v>2</v>
       </c>
@@ -3109,17 +3172,17 @@
       </c>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B4" s="164" t="s">
+      <c r="B4" s="175" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="165"/>
-      <c r="D4" s="166" t="s">
+      <c r="C4" s="176"/>
+      <c r="D4" s="177" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="168" t="s">
+      <c r="E4" s="179" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="170" t="s">
+      <c r="F4" s="181" t="s">
         <v>20</v>
       </c>
       <c r="G4" s="45"/>
@@ -3140,9 +3203,9 @@
       <c r="C5" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="167"/>
-      <c r="E5" s="169"/>
-      <c r="F5" s="171"/>
+      <c r="D5" s="178"/>
+      <c r="E5" s="180"/>
+      <c r="F5" s="182"/>
       <c r="L5" s="46">
         <v>4</v>
       </c>
@@ -3176,10 +3239,10 @@
       </c>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="174" t="s">
+      <c r="B7" s="160" t="s">
         <v>74</v>
       </c>
-      <c r="C7" s="175"/>
+      <c r="C7" s="161"/>
       <c r="D7" s="51" t="s">
         <v>33</v>
       </c>
@@ -3200,8 +3263,8 @@
       </c>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="176"/>
-      <c r="C8" s="177"/>
+      <c r="B8" s="162"/>
+      <c r="C8" s="163"/>
       <c r="D8" s="51" t="s">
         <v>38</v>
       </c>
@@ -3224,8 +3287,8 @@
       <c r="N8" s="48"/>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="176"/>
-      <c r="C9" s="177"/>
+      <c r="B9" s="162"/>
+      <c r="C9" s="163"/>
       <c r="D9" s="51" t="s">
         <v>43</v>
       </c>
@@ -3250,8 +3313,8 @@
       <c r="N9" s="55"/>
     </row>
     <row r="10" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="178"/>
-      <c r="C10" s="179"/>
+      <c r="B10" s="164"/>
+      <c r="C10" s="165"/>
       <c r="D10" s="56" t="s">
         <v>48</v>
       </c>
@@ -3284,19 +3347,19 @@
     <row r="12" spans="2:15" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="59"/>
       <c r="I12" s="46"/>
-      <c r="M12" s="172" t="s">
+      <c r="M12" s="158" t="s">
         <v>75</v>
       </c>
-      <c r="N12" s="173"/>
+      <c r="N12" s="159"/>
     </row>
     <row r="13" spans="2:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B13" s="158" t="s">
+      <c r="B13" s="166" t="s">
         <v>59</v>
       </c>
-      <c r="C13" s="159"/>
-      <c r="D13" s="159"/>
-      <c r="E13" s="159"/>
-      <c r="F13" s="160"/>
+      <c r="C13" s="167"/>
+      <c r="D13" s="167"/>
+      <c r="E13" s="167"/>
+      <c r="F13" s="168"/>
       <c r="M13" s="60" t="s">
         <v>25</v>
       </c>
@@ -3305,11 +3368,11 @@
       </c>
     </row>
     <row r="14" spans="2:15" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="161"/>
-      <c r="C14" s="162"/>
-      <c r="D14" s="162"/>
-      <c r="E14" s="162"/>
-      <c r="F14" s="163"/>
+      <c r="B14" s="169"/>
+      <c r="C14" s="170"/>
+      <c r="D14" s="170"/>
+      <c r="E14" s="170"/>
+      <c r="F14" s="171"/>
       <c r="M14" s="60" t="s">
         <v>30</v>
       </c>
@@ -3318,11 +3381,11 @@
       </c>
     </row>
     <row r="15" spans="2:15" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="180" t="s">
+      <c r="B15" s="172" t="s">
         <v>76</v>
       </c>
-      <c r="C15" s="180"/>
-      <c r="D15" s="180"/>
+      <c r="C15" s="172"/>
+      <c r="D15" s="172"/>
       <c r="E15" s="62" t="s">
         <v>60</v>
       </c>
@@ -3343,9 +3406,9 @@
       </c>
     </row>
     <row r="16" spans="2:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B16" s="181"/>
-      <c r="C16" s="181"/>
-      <c r="D16" s="181"/>
+      <c r="B16" s="173"/>
+      <c r="C16" s="173"/>
+      <c r="D16" s="173"/>
       <c r="E16" s="66"/>
       <c r="F16" s="51" t="s">
         <v>64</v>
@@ -3369,9 +3432,9 @@
       </c>
     </row>
     <row r="17" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="181"/>
-      <c r="C17" s="181"/>
-      <c r="D17" s="181"/>
+      <c r="B17" s="173"/>
+      <c r="C17" s="173"/>
+      <c r="D17" s="173"/>
       <c r="E17" s="66"/>
       <c r="F17" s="51" t="s">
         <v>67</v>
@@ -3395,9 +3458,9 @@
       </c>
     </row>
     <row r="18" spans="2:14" ht="14.45" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="181"/>
-      <c r="C18" s="181"/>
-      <c r="D18" s="181"/>
+      <c r="B18" s="173"/>
+      <c r="C18" s="173"/>
+      <c r="D18" s="173"/>
       <c r="E18" s="66"/>
       <c r="F18" s="51" t="s">
         <v>70</v>
@@ -3415,61 +3478,61 @@
       </c>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B19" s="181"/>
-      <c r="C19" s="181"/>
-      <c r="D19" s="181"/>
+      <c r="B19" s="173"/>
+      <c r="C19" s="173"/>
+      <c r="D19" s="173"/>
       <c r="E19" s="66"/>
-      <c r="F19" s="182" t="s">
+      <c r="F19" s="174" t="s">
         <v>78</v>
       </c>
-      <c r="G19" s="182"/>
+      <c r="G19" s="174"/>
     </row>
     <row r="20" spans="2:14" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="181"/>
-      <c r="C20" s="181"/>
-      <c r="D20" s="181"/>
+      <c r="B20" s="173"/>
+      <c r="C20" s="173"/>
+      <c r="D20" s="173"/>
       <c r="E20" s="66"/>
-      <c r="F20" s="182"/>
-      <c r="G20" s="182"/>
+      <c r="F20" s="174"/>
+      <c r="G20" s="174"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B21" s="181"/>
-      <c r="C21" s="181"/>
-      <c r="D21" s="181"/>
+      <c r="B21" s="173"/>
+      <c r="C21" s="173"/>
+      <c r="D21" s="173"/>
       <c r="E21" s="66"/>
-      <c r="F21" s="182"/>
-      <c r="G21" s="182"/>
+      <c r="F21" s="174"/>
+      <c r="G21" s="174"/>
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B22" s="181"/>
-      <c r="C22" s="181"/>
-      <c r="D22" s="181"/>
+      <c r="B22" s="173"/>
+      <c r="C22" s="173"/>
+      <c r="D22" s="173"/>
       <c r="E22" s="66"/>
-      <c r="F22" s="182"/>
-      <c r="G22" s="182"/>
+      <c r="F22" s="174"/>
+      <c r="G22" s="174"/>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B23" s="181"/>
-      <c r="C23" s="181"/>
-      <c r="D23" s="181"/>
+      <c r="B23" s="173"/>
+      <c r="C23" s="173"/>
+      <c r="D23" s="173"/>
       <c r="E23" s="66"/>
-      <c r="F23" s="182"/>
-      <c r="G23" s="182"/>
+      <c r="F23" s="174"/>
+      <c r="G23" s="174"/>
     </row>
     <row r="25" spans="2:14" ht="17.45" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="OpD0C6psjTe/kStoo1h7yvA+15jkxfWm/NBH5QdNDZMthMHZ8e+D8fccabo00cUHiBPBG012UpwlWS/LhPlnkg==" saltValue="T+6KfbnqR49JhNBhr/3oaA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="10">
+    <mergeCell ref="B2:F3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
     <mergeCell ref="M12:N12"/>
     <mergeCell ref="B7:C10"/>
     <mergeCell ref="B13:F14"/>
     <mergeCell ref="B15:D23"/>
     <mergeCell ref="F19:G23"/>
-    <mergeCell ref="B2:F3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F4:F5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3524,15 +3587,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002C289946819CFF499E91D197BC975371" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="674b7a4e239a9748c7aaa97e309327a4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cca9fd2d-ef84-45c9-8063-8f4bd4c29606" xmlns:ns3="18557d39-01b8-4d71-9479-3fad465290ae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="600253478e594d1349e02792803dc53a" ns2:_="" ns3:_="">
     <xsd:import namespace="cca9fd2d-ef84-45c9-8063-8f4bd4c29606"/>
@@ -3749,6 +3803,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3760,14 +3823,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42C52D6A-E0AB-44E7-ABE4-D928B05D246F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A2CE780C-3974-4A71-8F18-23A7FE356660}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3786,6 +3841,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42C52D6A-E0AB-44E7-ABE4-D928B05D246F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4FB4873-1F2B-4DA5-A59D-EA2845F46BB6}">
   <ds:schemaRefs>

</xml_diff>